<commit_message>
Use the English font name in the reference workbook
Replace the localized theme font name with Malgun Gothic without changing workbook data.
</commit_message>
<xml_diff>
--- a/xrd_dashboard/resources/ReferencePeaks.xlsx
+++ b/xrd_dashboard/resources/ReferencePeaks.xlsx
@@ -171,7 +171,7 @@
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hang" typeface="Malgun Gothic"/>
         <a:font script="Hans" typeface="等线 Light"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Times New Roman"/>
@@ -223,7 +223,7 @@
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hang" typeface="Malgun Gothic"/>
         <a:font script="Hans" typeface="等线"/>
         <a:font script="Hant" typeface="新細明體"/>
         <a:font script="Arab" typeface="Arial"/>

</xml_diff>